<commit_message>
feat(gameplay): advance StackCraft foundation parity
Static checks passed: git diff --check, spec-lint, spec-lint tests, unity-yaml-guard, gameplay-static-preflight, stackcraft-business-representative-audit.

Known gap: EditMode batch test currently fails with 27 failing tests out of 580 after user approval to push anyway.
</commit_message>
<xml_diff>
--- a/EX_GAS_Config/ProjectConfigTable/exgas_config/Datas/#exgas.gameplayTags.xlsx
+++ b/EX_GAS_Config/ProjectConfigTable/exgas_config/Datas/#exgas.gameplayTags.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19" customWidth="1" min="3" max="3"/>
@@ -1046,6 +1046,201 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="B41" t="n">
+        <v>800</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>卡牌语义标签</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" t="n">
+        <v>8001</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Card.Category</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>卡牌类别</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" t="n">
+        <v>8001001</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Card.Category.Resource</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>卡牌类别：资源</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" t="n">
+        <v>8001002</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Card.Category.Character</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>卡牌类别：角色</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" t="n">
+        <v>8001003</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Card.Category.Consumable</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>卡牌类别：消耗品</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" t="n">
+        <v>8001004</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Card.Category.Material</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>卡牌类别：材料</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" t="n">
+        <v>8001005</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Card.Category.Equipment</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>卡牌类别：装备</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" t="n">
+        <v>8001006</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Card.Category.Structure</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>卡牌类别：建筑</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" t="n">
+        <v>8001007</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Card.Category.Currency</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>卡牌类别：货币</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" t="n">
+        <v>8001008</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Card.Category.Recipe</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>卡牌类别：配方</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" t="n">
+        <v>8001009</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Card.Category.Mob</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>卡牌类别：生物/敌对单位</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" t="n">
+        <v>8001010</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Card.Category.Area</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>卡牌类别：地区</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" t="n">
+        <v>8001011</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Card.Category.Valuable</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>卡牌类别：贵重物</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>